<commit_message>
feat: layout sidebar updates & notifikasi
</commit_message>
<xml_diff>
--- a/public/templates/template_surat_jalan.xlsx
+++ b/public/templates/template_surat_jalan.xlsx
@@ -15,66 +15,69 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="20">
-  <si>
-    <t>tanggal</t>
-  </si>
-  <si>
-    <t>nama_barang</t>
-  </si>
-  <si>
-    <t>volume_keluar</t>
-  </si>
-  <si>
-    <t>no_polisi</t>
-  </si>
-  <si>
-    <t>lokasi</t>
-  </si>
-  <si>
-    <t>pemohon</t>
-  </si>
-  <si>
-    <t>petugas</t>
-  </si>
-  <si>
-    <t>no_surat_jalan</t>
-  </si>
-  <si>
-    <t>kecamatan_pelaksana</t>
-  </si>
-  <si>
-    <t>keterangan</t>
-  </si>
-  <si>
-    <t>15 Januari 2026</t>
-  </si>
-  <si>
-    <t>TRIPLEK/MULTIPLEK</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="21">
+  <si>
+    <t>Tanggal</t>
+  </si>
+  <si>
+    <t>Nama Barang</t>
+  </si>
+  <si>
+    <t>Volume Keluar</t>
+  </si>
+  <si>
+    <t>No. Polisi</t>
+  </si>
+  <si>
+    <t>Lokasi Tujuan</t>
+  </si>
+  <si>
+    <t>Pemohon</t>
+  </si>
+  <si>
+    <t>Petugas (Admin)</t>
+  </si>
+  <si>
+    <t>Penerima Barang</t>
+  </si>
+  <si>
+    <t>No. Surat Jalan</t>
+  </si>
+  <si>
+    <t>Kecamatan / Pelaksana</t>
+  </si>
+  <si>
+    <t>Keterangan</t>
+  </si>
+  <si>
+    <t>30/04/2026</t>
+  </si>
+  <si>
+    <t>BATU PECAH 2/3</t>
   </si>
   <si>
     <t>B 1234 ABC</t>
   </si>
   <si>
-    <t>POMPA SINDANG</t>
-  </si>
-  <si>
-    <t>SHOLAHUDDIN</t>
-  </si>
-  <si>
-    <t>Sanjaya</t>
-  </si>
-  <si>
-    <t>90/GKU/I/2026</t>
-  </si>
-  <si>
-    <t>PEMELIHARAAN</t>
-  </si>
-  <si>
-    <t>Inventaris</t>
-  </si>
-  <si>
-    <t>PAKU 2"-5"</t>
+    <t>Lokasi Proyek A</t>
+  </si>
+  <si>
+    <t>Bpk. Ahmad</t>
+  </si>
+  <si>
+    <t>SANJAYA</t>
+  </si>
+  <si>
+    <t>Sdr. Budi</t>
+  </si>
+  <si>
+    <t>SJ-20260430-001</t>
+  </si>
+  <si>
+    <t>Kec. Gambir</t>
+  </si>
+  <si>
+    <t>Catatan tambahan jika ada</t>
   </si>
 </sst>
 </file>
@@ -82,7 +85,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <b val="0"/>
       <i val="0"/>
@@ -92,16 +95,35 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <b val="1"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <gradientFill type="linear" degree="90">
+        <stop position="0">
+          <color rgb="FFA0A0A0"/>
+        </stop>
+        <stop position="1">
+          <color rgb="FFFFFFFF"/>
+        </stop>
+      </gradientFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -109,12 +131,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="1" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="2" borderId="2" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -414,115 +466,89 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="18.71" bestFit="true" customWidth="true" style="0"/>
-    <col min="2" max="2" width="21.138" bestFit="true" customWidth="true" style="0"/>
-    <col min="3" max="3" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="4" max="4" width="12.854" bestFit="true" customWidth="true" style="0"/>
-    <col min="5" max="5" width="16.425" bestFit="true" customWidth="true" style="0"/>
-    <col min="6" max="6" width="13.997" bestFit="true" customWidth="true" style="0"/>
-    <col min="7" max="7" width="9.283" bestFit="true" customWidth="true" style="0"/>
-    <col min="8" max="8" width="17.567" bestFit="true" customWidth="true" style="0"/>
-    <col min="9" max="9" width="23.423" bestFit="true" customWidth="true" style="0"/>
-    <col min="10" max="10" width="12.854" bestFit="true" customWidth="true" style="0"/>
+    <col min="1" max="1" width="12.854" customWidth="true" style="0"/>
+    <col min="2" max="2" width="17.567" customWidth="true" style="0"/>
+    <col min="3" max="3" width="18.71" customWidth="true" style="0"/>
+    <col min="4" max="4" width="15.139" customWidth="true" style="0"/>
+    <col min="5" max="5" width="18.71" customWidth="true" style="0"/>
+    <col min="6" max="6" width="12.854" customWidth="true" style="0"/>
+    <col min="7" max="7" width="20.995" customWidth="true" style="0"/>
+    <col min="9" max="9" width="20.995" customWidth="true" style="0"/>
+    <col min="10" max="10" width="28.136" customWidth="true" style="0"/>
+    <col min="11" max="11" width="30.564" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
-      <c r="A1" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
+      <c r="K1" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2">
-        <v>2</v>
-      </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="J2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
         <v>19</v>
       </c>
-      <c r="C3">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G3" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
-      <c r="J3" t="s">
-        <v>18</v>
+      <c r="K2" t="s">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>